<commit_message>
auto: snapshot 2026-09-13 13:31:02
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -50620,7 +50620,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-13 13:01:00</t>
+          <t>Timestamp: 2026-09-13 13:31:00</t>
         </is>
       </c>
     </row>
@@ -51368,11 +51368,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>44877</v>
+        <v>45045</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+6792</t>
+          <t>+6960</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-19 13:31:02
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -55900,7 +55900,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-19 13:01:00</t>
+          <t>Timestamp: 2026-09-19 13:31:00</t>
         </is>
       </c>
     </row>
@@ -56198,11 +56198,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>2268</v>
+        <v>2352</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>+98</t>
         </is>
       </c>
     </row>
@@ -56633,11 +56633,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>72269</v>
+        <v>72383</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+3935</t>
+          <t>+4049</t>
         </is>
       </c>
     </row>
@@ -56678,11 +56678,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>9630</v>
+        <v>9667</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1473</t>
+          <t>+1510</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-20 13:31:01
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -56780,7 +56780,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-20 13:01:00</t>
+          <t>Timestamp: 2026-09-20 13:31:00</t>
         </is>
       </c>
     </row>
@@ -57074,7 +57074,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>SeeYouSoon</t>
+          <t>SNC | Asuna</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
@@ -57082,7 +57082,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+23640</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>